<commit_message>
Upload adaptive campus case study dataset
</commit_message>
<xml_diff>
--- a/campus_cases.xlsx
+++ b/campus_cases.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
   <si>
     <t>Case</t>
   </si>
@@ -289,6 +289,105 @@
   </si>
   <si>
     <t>manufacturing reuse, transparency, industrial campus</t>
+  </si>
+  <si>
+    <t>TU Delft BK City</t>
+  </si>
+  <si>
+    <t>Former chemistry faculty building</t>
+  </si>
+  <si>
+    <t>Architecture faculty / built environment campus</t>
+  </si>
+  <si>
+    <t>Large historic campus building, long corridors, flexible studio spaces, reused lecture halls and public interior streets</t>
+  </si>
+  <si>
+    <t>adaptive reuse, campus renewal, studio, corridor, historic integration, flexible learning</t>
+  </si>
+  <si>
+    <t>Netherlands</t>
+  </si>
+  <si>
+    <t>2008/2009</t>
+  </si>
+  <si>
+    <t>Delft</t>
+  </si>
+  <si>
+    <t>Europe</t>
+  </si>
+  <si>
+    <t>University of Toronto Daniels Building</t>
+  </si>
+  <si>
+    <t>Knox College / theological college</t>
+  </si>
+  <si>
+    <t>Architecture, landscape and design faculty</t>
+  </si>
+  <si>
+    <t>Gothic heritage building integrated with contemporary addition, circular urban site, studios, library, public programming spaces</t>
+  </si>
+  <si>
+    <t>heritage reuse, architecture school, studio, public programming, historic integration, campus gateway</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>2017</t>
+  </si>
+  <si>
+    <t>Toronto</t>
+  </si>
+  <si>
+    <t>North America</t>
+  </si>
+  <si>
+    <t>Duke University Smith Warehouse</t>
+  </si>
+  <si>
+    <t>Tobacco warehouse</t>
+  </si>
+  <si>
+    <t>University arts spaces and offices</t>
+  </si>
+  <si>
+    <t>Industrial warehouse shell, large open floor plates, arts studios, office bays, campus-city interface</t>
+  </si>
+  <si>
+    <t>industrial reuse, warehouse, arts campus, large-span, studio, public connectivity</t>
+  </si>
+  <si>
+    <t>2011</t>
+  </si>
+  <si>
+    <t>Durham, North Carolina</t>
+  </si>
+  <si>
+    <t>Aalto University Harald Herlin Learning Centre</t>
+  </si>
+  <si>
+    <t>Helsinki University of Technology main library</t>
+  </si>
+  <si>
+    <t>Learning centre / library services</t>
+  </si>
+  <si>
+    <t>Renovated Aalto-designed library, indirect daylight, fan-like plan, study and groupwork spaces, exhibition spaces, cafe</t>
+  </si>
+  <si>
+    <t>library renewal, daylight, flexible learning, exhibition, campus publicness, historic integration</t>
+  </si>
+  <si>
+    <t>Finland</t>
+  </si>
+  <si>
+    <t>2016</t>
+  </si>
+  <si>
+    <t>Espoo</t>
   </si>
 </sst>
 </file>
@@ -552,7 +651,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
@@ -955,20 +1054,120 @@
       <c r="J17" s="5"/>
     </row>
     <row r="18">
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
+      <c r="A18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" t="s">
+        <v>93</v>
+      </c>
+      <c r="D18" t="s">
+        <v>94</v>
+      </c>
+      <c r="E18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F18" t="s">
+        <v>96</v>
+      </c>
+      <c r="G18" t="s">
+        <v>97</v>
+      </c>
+      <c r="H18" t="s">
+        <v>98</v>
+      </c>
+      <c r="I18" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="19">
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
+      <c r="A19" t="s">
+        <v>100</v>
+      </c>
+      <c r="B19" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" t="s">
+        <v>103</v>
+      </c>
+      <c r="E19" t="s">
+        <v>104</v>
+      </c>
+      <c r="F19" t="s">
+        <v>105</v>
+      </c>
+      <c r="G19" t="s">
+        <v>106</v>
+      </c>
+      <c r="H19" t="s">
+        <v>107</v>
+      </c>
+      <c r="I19" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="20">
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
+      <c r="A20" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C20" t="s">
+        <v>111</v>
+      </c>
+      <c r="D20" t="s">
+        <v>112</v>
+      </c>
+      <c r="E20" t="s">
+        <v>113</v>
+      </c>
+      <c r="F20" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" t="s">
+        <v>114</v>
+      </c>
+      <c r="H20" t="s">
+        <v>115</v>
+      </c>
+      <c r="I20" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
+      <c r="A21" t="s">
+        <v>116</v>
+      </c>
+      <c r="B21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C21" t="s">
+        <v>118</v>
+      </c>
+      <c r="D21" t="s">
+        <v>119</v>
+      </c>
+      <c r="E21" t="s">
+        <v>120</v>
+      </c>
+      <c r="F21" t="s">
+        <v>121</v>
+      </c>
+      <c r="G21" t="s">
+        <v>122</v>
+      </c>
+      <c r="H21" t="s">
+        <v>123</v>
+      </c>
+      <c r="I21" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="I22" s="5"/>
@@ -4888,26 +5087,26 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A2"/>
-    <hyperlink r:id="rId2" ref="A3"/>
-    <hyperlink r:id="rId3" ref="A4"/>
-    <hyperlink r:id="rId4" ref="A5"/>
-    <hyperlink r:id="rId5" ref="A6"/>
-    <hyperlink r:id="rId6" ref="A7"/>
-    <hyperlink r:id="rId7" ref="A8"/>
-    <hyperlink r:id="rId8" ref="A9"/>
-    <hyperlink r:id="rId9" ref="A10"/>
-    <hyperlink r:id="rId10" ref="A11"/>
-    <hyperlink r:id="rId11" ref="A12"/>
-    <hyperlink r:id="rId12" ref="A13"/>
-    <hyperlink r:id="rId13" ref="A14"/>
-    <hyperlink r:id="rId14" ref="A15"/>
-    <hyperlink r:id="rId15" ref="A16"/>
-    <hyperlink r:id="rId16" ref="A17"/>
+    <hyperlink ns1:id="rId1" ref="A2"/>
+    <hyperlink ns1:id="rId2" ref="A3"/>
+    <hyperlink ns1:id="rId3" ref="A4"/>
+    <hyperlink ns1:id="rId4" ref="A5"/>
+    <hyperlink ns1:id="rId5" ref="A6"/>
+    <hyperlink ns1:id="rId6" ref="A7"/>
+    <hyperlink ns1:id="rId7" ref="A8"/>
+    <hyperlink ns1:id="rId8" ref="A9"/>
+    <hyperlink ns1:id="rId9" ref="A10"/>
+    <hyperlink ns1:id="rId10" ref="A11"/>
+    <hyperlink ns1:id="rId11" ref="A12"/>
+    <hyperlink ns1:id="rId12" ref="A13"/>
+    <hyperlink ns1:id="rId13" ref="A14"/>
+    <hyperlink ns1:id="rId14" ref="A15"/>
+    <hyperlink ns1:id="rId15" ref="A16"/>
+    <hyperlink ns1:id="rId16" ref="A17"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId17"/>
+  <drawing ns1:id="rId17"/>
 </worksheet>
 </file>
</xml_diff>